<commit_message>
feat: foto SortItOutSi reali per le 4 seconde squadre IT3 (106 match DOB-verificati, 105 IT3 con face)
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_dob_mismatch.xlsx
+++ b/data/sots_more_matches_dob_mismatch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -485,7 +485,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>New arrival</t>
+          <t>Frosinone Primavera</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Winter signing</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -606,86 +606,86 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alessandro Marcandalli</t>
+          <t>Alessio Sibilano</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>818448</v>
+        <v>1168030</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Returnee</t>
+          <t>Sassuolo Primavera</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2002-10-25</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2002-02-25</t>
+          <t>2007-07-06</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>43500463</v>
+        <v>2000268216</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>alessandro-marcandalli</t>
+          <t>alessio-sibilano</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Genoa CFC</t>
+          <t>US Sassuolo</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43500463/alessandro-marcandalli</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000268216/alessio-sibilano</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alessio Sibilano</t>
+          <t>Alfonso De Luca</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1168030</v>
+        <v>1077899</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Internal transfer: Sassuolo Under 18; date: 01/07/2025</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2006-09-19</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2007-07-06</t>
+          <t>2006-06-19</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2000268216</v>
+        <v>2000242306</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>alessio-sibilano</t>
+          <t>alfonso-de-luca</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>SSC Napoli</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268216/alessio-sibilano</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000242306/alfonso-de-luca</t>
         </is>
       </c>
     </row>
@@ -710,11 +710,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2006-06-19</t>
+          <t>1997-07-14</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2000242306</v>
+        <v>2000427316</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -723,70 +723,70 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SSC Napoli</t>
+          <t>US Avellino 1912</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000242306/alfonso-de-luca</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000427316/alfonso-de-luca</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alfonso De Luca</t>
+          <t>Andrea Campani</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1077899</v>
+        <v>1044819</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Napoli Primavera</t>
+          <t>Sassuolo Primavera</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2006-09-19</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1997-07-14</t>
+          <t>2007-04-03</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2000427316</v>
+        <v>2000268200</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>alfonso-de-luca</t>
+          <t>andrea-campani</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>US Avellino 1912</t>
+          <t>US Sassuolo</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000427316/alfonso-de-luca</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000268200/andrea-campani</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Andrea Campani</t>
+          <t>Andrea Caucci</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1044819</v>
+        <v>1051116</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Internal transfer: Sassuolo Under 18; date: 01/07/2025</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -796,40 +796,40 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2007-04-03</t>
+          <t>2007-06-30</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2000268200</v>
+        <v>2000266831</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>andrea-campani</t>
+          <t>andrea-caucci</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>SSC Napoli</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268200/andrea-campani</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000266831/andrea-caucci</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Andrea Caucci</t>
+          <t>Andrea Lantignotti</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1051116</v>
+        <v>1296425</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Napoli Primavera</t>
+          <t>Cesena Primavera</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -839,40 +839,40 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2007-06-30</t>
+          <t>2007-05-31</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2000266831</v>
+        <v>2000284355</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>andrea-caucci</t>
+          <t>andrea-lantignotti</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SSC Napoli</t>
+          <t>Cesena FC</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266831/andrea-caucci</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000284355/andrea-lantignotti</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Andrea Lantignotti</t>
+          <t>Bruno Zorzetto</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1296425</v>
+        <v>1182950</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Internal transfer: Cesena Under 18; date: 01/07/2025</t>
+          <t>Frosinone Primavera</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -882,144 +882,144 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2007-05-31</t>
+          <t>2007-12-21</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2000284355</v>
+        <v>2000495913</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>andrea-lantignotti</t>
+          <t>bruno-zorzetto</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Cesena FC</t>
+          <t>Frosinone Calcio</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284355/andrea-lantignotti</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000495913/bruno-zorzetto</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bruno Zorzetto</t>
+          <t>Bryant Nieling</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1182950</v>
+        <v>698082</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Internal transfer: Frosinone Under 18; date: 01/07/2025</t>
+          <t>Modena FC</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2002-10-31</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2007-12-21</t>
+          <t>2001-11-30</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2000495913</v>
+        <v>2000017548</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>bruno-zorzetto</t>
+          <t>bryant-nieling</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Frosinone Calcio</t>
+          <t>Modena FC</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495913/bruno-zorzetto</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000017548/bryant-nieling</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bryant Nieling</t>
+          <t>Catello Amendola</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>698082</v>
+        <v>1133143</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>New arrival</t>
+          <t>Sassuolo Primavera</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2002-10-31</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2001-11-30</t>
+          <t>2007-02-04</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2000017548</v>
+        <v>2000268221</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>bryant-nieling</t>
+          <t>catello-amendola</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Modena FC</t>
+          <t>US Sassuolo</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000017548/bryant-nieling</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000268221/catello-amendola</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Catello Amendola</t>
+          <t>Diego Tampieri</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1133143</v>
+        <v>1129564</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Internal transfer: Sassuolo Under 18; date: 01/07/2025</t>
+          <t>Sassuolo Primavera</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2006-01-25</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2007-02-04</t>
+          <t>2006-01-01</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2000268221</v>
+        <v>2000187279</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>catello-amendola</t>
+          <t>diego-tampieri</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1029,70 +1029,70 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268221/catello-amendola</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000187279/diego-tampieri</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Daniel Theiner</t>
+          <t>Divine Onyemachi</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>886189</v>
+        <v>1117532</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Returnee</t>
+          <t>Lecce Primavera</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2004-02-25</t>
+          <t>2007-08-02</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2004-02-26</t>
+          <t>2006-12-13</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2000098802</v>
+        <v>2000307954</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>daniel-theiner</t>
+          <t>divine-onyemachi</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>FC Südtirol</t>
+          <t>US Lecce</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000098802/daniel-theiner</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000307954/divine-onyemachi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>David Odogu</t>
+          <t>Eddy Kouadio</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>897423</v>
+        <v>957822</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New arrival</t>
+          <t>Fiorentina Primavera</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2006-06-03</t>
+          <t>2006-05-07</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1101,140 +1101,140 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2000218552</v>
+        <v>2000184141</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>david-odogu</t>
+          <t>eddy-kouadio</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>ACF Fiorentina</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000218552/david-odogu</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000184141/eddy-kouadio</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Diego Tampieri</t>
+          <t>Emilio Amadori</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1129564</v>
+        <v>1296435</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>New arrival</t>
+          <t>Cesena Primavera</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2006-01-25</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2006-01-01</t>
+          <t>2007-01-08</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2000187279</v>
+        <v>2000284319</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>diego-tampieri</t>
+          <t>emilio-amadori</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Cesena FC</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000187279/diego-tampieri</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000284319/emilio-amadori</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Divine Onyemachi</t>
+          <t>Francesco Leone</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1117532</v>
+        <v>1182369</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>New arrival</t>
+          <t>Juventus Primavera</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2007-08-02</t>
+          <t>2007-05-03</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2006-12-13</t>
+          <t>2007-05-30</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2000307954</v>
+        <v>2000332032</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>divine-onyemachi</t>
+          <t>francesco-leone</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>US Lecce</t>
+          <t>Juventus FC</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000307954/divine-onyemachi</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000332032/francesco-leone</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Eddy Kouadio</t>
+          <t>Gianmaria Fei</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>957822</v>
+        <v>1317913</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Internal transfer: Fiorentina Primavera; date: 01/07/2025</t>
+          <t>Fiorentina Primavera</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2006-05-07</t>
+          <t>2007-04-15</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2006-05-03</t>
+          <t>2007-04-17</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2000184141</v>
+        <v>2000403058</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>eddy-kouadio</t>
+          <t>gianmaria-fei</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1244,212 +1244,212 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000184141/eddy-kouadio</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000403058/gianmaria-fei</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Emanuele Adamo</t>
+          <t>Giovanni Andrea Cardu</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>411666</v>
+        <v>1253653</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Winter signing</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1998-07-19</t>
+          <t>2008-05-11</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1998-06-19</t>
+          <t>2008-05-19</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>43272168</v>
+        <v>2000461316</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>emanuele-adamo</t>
+          <t>giovanni-andrea-cardu</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Spezia Calcio</t>
+          <t>Cagliari Calcio</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43272168/emanuele-adamo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000461316/giovanni-andrea-cardu</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Emilio Amadori</t>
+          <t>Ioan Vermeșan</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1296435</v>
+        <v>928037</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Internal transfer: Cesena Under 18; date: 01/07/2025</t>
+          <t>Hellas Verona Primavera</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2006-10-18</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2007-01-08</t>
+          <t>2006-10-15</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2000284319</v>
+        <v>2000157324</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>emilio-amadori</t>
+          <t>ioan-vermesan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Cesena FC</t>
+          <t>Hellas Verona</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284319/emilio-amadori</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000157324/ioan-vermesan</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Francesco Leone</t>
+          <t>Isaac Enoghama</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1182369</v>
+        <v>1075420</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Returnee</t>
+          <t>Genoa Primavera</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2007-05-03</t>
+          <t>2007-09-10</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2007-05-30</t>
+          <t>2007-08-10</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2000332032</v>
+        <v>2000266435</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>francesco-leone</t>
+          <t>isaac-enoghama</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Juventus FC</t>
+          <t>Genoa CFC</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000332032/francesco-leone</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000266435/isaac-enoghama</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gianmaria Fei</t>
+          <t>Jack Nunn</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1317913</v>
+        <v>1292591</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Internal transfer: Fiorentina Under 18; date: 01/07/2025</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2007-04-15</t>
+          <t>2006-07-07</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2007-04-17</t>
+          <t>2006-07-08</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2000403058</v>
+        <v>2000389422</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>gianmaria-fei</t>
+          <t>jack-nunn</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>ACF Fiorentina</t>
+          <t>Cagliari Calcio</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000403058/gianmaria-fei</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000389422/jack-nunn</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Giovanni Andrea Cardu</t>
+          <t>Joseph Liteta</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1253653</v>
+        <v>1134304</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Internal transfer: Cagliari Under 17; date: 01/07/2025</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2008-05-11</t>
+          <t>2006-02-22</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2008-05-19</t>
+          <t>2006-01-22</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2000461316</v>
+        <v>2000241198</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>giovanni-andrea-cardu</t>
+          <t>joseph-liteta</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1459,710 +1459,710 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000461316/giovanni-andrea-cardu</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000241198/joseph-liteta</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Henrik Meister</t>
+          <t>Lorenzo Nyarko</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>914934</v>
+        <v>1168024</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>New arrival</t>
+          <t>Sassuolo Primavera</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2003-11-13</t>
+          <t>2007-10-20</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2003-11-17</t>
+          <t>2007-08-20</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2000113465</v>
+        <v>2000268210</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>henrik-meister</t>
+          <t>lorenzo-nyarko</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Pisa Sporting Club</t>
+          <t>US Sassuolo</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000113465/henrik-meister</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000268210/lorenzo-nyarko</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ioan Vermeșan</t>
+          <t>Lorenzo Pio Marino</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>928037</v>
+        <v>1100015</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hellas Verona Primavera</t>
+          <t>Cremonese Primavera</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2006-10-18</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2006-10-15</t>
+          <t>2007-01-03</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2000157324</v>
+        <v>2000261855</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>ioan-vermesan</t>
+          <t>lorenzo-pio-marino</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Hellas Verona</t>
+          <t>US Cremonese</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000157324/ioan-vermesan</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000261855/lorenzo-pio-marino</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Isaac Enoghama</t>
+          <t>Luca Gobbo</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1075420</v>
+        <v>1183953</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Internal transfer: Genoa Under 18; date: 01/07/2025</t>
+          <t>Atalanta Primavera</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2007-09-10</t>
+          <t>2006-04-05</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2007-08-10</t>
+          <t>2006-04-07</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2000266435</v>
+        <v>2000333546</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>isaac-enoghama</t>
+          <t>luca-gobbo</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Genoa CFC</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266435/isaac-enoghama</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000333546/luca-gobbo</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jack Nunn</t>
+          <t>Ludovico Varali</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1292591</v>
+        <v>1388316</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Cagliari Primavera</t>
+          <t>Parma Primavera</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2006-07-07</t>
+          <t>2009-01-17</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2006-07-08</t>
+          <t>2009-01-06</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2000389422</v>
+        <v>2000491914</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>jack-nunn</t>
+          <t>ludovico-varali</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000389422/jack-nunn</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000491914/ludovico-varali</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Joseph Liteta</t>
+          <t>Marco Tiozzo</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1134304</v>
+        <v>1234457</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Internal transfer: Cagliari Primavera; date: 19/10/2025</t>
+          <t>Juventus Primavera</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2006-02-22</t>
+          <t>2008-10-07</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2006-01-22</t>
+          <t>2008-07-10</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2000241198</v>
+        <v>2000386592</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>joseph-liteta</t>
+          <t>marco-tiozzo-pagio</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Juventus FC</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000241198/joseph-liteta</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000386592/marco-tiozzo-pagio</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Lorenzo Nyarko</t>
+          <t>Mariano Troilo</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1168024</v>
+        <v>1159864</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2007-10-20</t>
+          <t>2003-06-28</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2007-08-20</t>
+          <t>2003-06-22</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2000268210</v>
+        <v>2000200406</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>lorenzo-nyarko</t>
+          <t>mariano-troilo</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268210/lorenzo-nyarko</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000200406/mariano-troilo</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Lorenzo Pio Marino</t>
+          <t>Mark Topollaj</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1100015</v>
+        <v>949340</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Cremonese Primavera</t>
+          <t>Hellas Verona Primavera</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2007-09-25</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2007-01-03</t>
+          <t>2007-08-25</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>2000261855</v>
+        <v>2000269202</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>lorenzo-pio-marino</t>
+          <t>mark-topollaj</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>US Cremonese</t>
+          <t>Hellas Verona</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000261855/lorenzo-pio-marino</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000269202/mark-topollaj</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Luca Gobbo</t>
+          <t>Marko Farji</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1183953</v>
+        <v>663153</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Atalanta Primavera</t>
+          <t>Venezia FC</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2006-04-05</t>
+          <t>2004-03-16</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2006-04-07</t>
+          <t>2004-03-26</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2000333546</v>
+        <v>2000065330</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>luca-gobbo</t>
+          <t>marko-farji</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Atalanta BC</t>
+          <t>Venezia FC</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000333546/luca-gobbo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000065330/marko-farji</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ludovico Varali</t>
+          <t>Márton Prettenhoffer</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1388316</v>
+        <v>1060896</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Parma Primavera</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2009-01-17</t>
+          <t>2008-03-10</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2009-01-06</t>
+          <t>2008-03-17</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2000491914</v>
+        <v>2000394155</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>ludovico-varali</t>
+          <t>marton-prettenhoffer</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Cagliari Calcio</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000491914/ludovico-varali</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000394155/marton-prettenhoffer</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Marco Romano</t>
+          <t>Mattia Aliprandi</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>902615</v>
+        <v>1170819</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Genoa U20</t>
+          <t>Atalanta Primavera</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2006-03-01</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1985-06-17</t>
+          <t>2007-01-04</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>43023299</v>
+        <v>2000330730</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>marco-romano</t>
+          <t>mattia-aliprandi</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>SSC Napoli</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43023299/marco-romano</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000330730/mattia-aliprandi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Marco Sala</t>
+          <t>Michael Zeppieri</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>392570</v>
+        <v>1084276</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Winter signing</t>
+          <t>Torino Primavera</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1999-06-04</t>
+          <t>2006-06-01</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1971-09-16</t>
+          <t>2006-09-23</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>43269015</v>
+        <v>2000269983</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>marco-sala</t>
+          <t>michael-zeppieri</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Inter Milan</t>
+          <t>Torino FC</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43269015/marco-sala</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000269983/michael-zeppieri</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marco Tiozzo</t>
+          <t>Noe Mael Tagne</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1234457</v>
+        <v>1310290</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Internal transfer: Juventus Under 17; date: 01/07/2025</t>
+          <t>Hellas Verona Primavera</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2008-10-07</t>
+          <t>2008-08-08</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2008-07-10</t>
+          <t>2008-08-11</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2000386592</v>
+        <v>2000400138</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>marco-tiozzo-pagio</t>
+          <t>noe-mael-tagne</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Juventus FC</t>
+          <t>Hellas Verona</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000386592/marco-tiozzo-pagio</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000400138/noe-mael-tagne</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Mariano Troilo</t>
+          <t>Noham Hamdaoua</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1159864</v>
+        <v>1295337</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>New arrival</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2003-06-28</t>
+          <t>2007-12-16</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2003-06-22</t>
+          <t>2007-01-17</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2000200406</v>
+        <v>2000382032</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>mariano-troilo</t>
+          <t>noham-hamdaoua</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Cagliari Calcio</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000200406/mariano-troilo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000382032/noham-hamdaoua</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mark Topollaj</t>
+          <t>Piergiorgio Bonanno</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>949340</v>
+        <v>1190028</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Internal transfer: Hellas Verona Under 18; date: 01/07/2025</t>
+          <t>Fiorentina Primavera</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2007-09-25</t>
+          <t>2007-06-27</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2007-08-25</t>
+          <t>2007-06-26</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2000269202</v>
+        <v>2000333018</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>mark-topollaj</t>
+          <t>piergiorgio-bonanno</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Hellas Verona</t>
+          <t>ACF Fiorentina</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000269202/mark-topollaj</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000333018/piergiorgio-bonanno</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Marko Farji</t>
+          <t>Raffaele Colella</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>663153</v>
+        <v>1318329</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Winter signing</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2004-03-16</t>
+          <t>2006-05-01</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2004-03-26</t>
+          <t>2006-05-04</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2000065330</v>
+        <v>2000266816</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>marko-farji</t>
+          <t>raffaele-colella</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Venezia FC</t>
+          <t>SSC Napoli</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000065330/marko-farji</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000266816/raffaele-colella</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Márton Prettenhoffer</t>
+          <t>Riccardo Biguzzi</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1060896</v>
+        <v>1296430</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Cagliari Primavera</t>
+          <t>Cesena Primavera</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2008-03-10</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2008-03-17</t>
+          <t>2007-02-06</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>2000394155</v>
+        <v>2000284347</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>marton-prettenhoffer</t>
+          <t>riccardo-biguzzi</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Cesena FC</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000394155/marton-prettenhoffer</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000284347/riccardo-biguzzi</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mattia Aliprandi</t>
+          <t>Salvatore De Martino</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1170819</v>
+        <v>1440090</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Internal transfer: Atalanta Under 18; date: 01/07/2025</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2172,122 +2172,122 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2007-01-04</t>
+          <t>2007-09-24</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>2000330730</v>
+        <v>2000266709</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>mattia-aliprandi</t>
+          <t>salvatore-de-martino</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Atalanta BC</t>
+          <t>SSC Napoli</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000330730/mattia-aliprandi</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000266709/salvatore-de-martino</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Michael Zeppieri</t>
+          <t>Tommaso Reali</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1084276</v>
+        <v>1311736</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Torino Primavera</t>
+          <t>Frosinone Primavera</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2006-06-01</t>
+          <t>2008-03-25</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2006-09-23</t>
+          <t>2008-01-01</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>2000269983</v>
+        <v>2000495914</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>michael-zeppieri</t>
+          <t>tommaso-reali</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Torino FC</t>
+          <t>Frosinone Calcio</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000269983/michael-zeppieri</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000495914/tommaso-reali</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Noe Mael Tagne</t>
+          <t>Vincenzo Testa</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1310290</v>
+        <v>1243102</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Internal transfer: Hellas Under 17; date: 01/07/2025</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2008-08-08</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2008-08-11</t>
+          <t>2007-01-01</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>2000400138</v>
+        <v>2000495803</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>noe-mael-tagne</t>
+          <t>vincenzo-testa</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Hellas Verona</t>
+          <t>SSC Napoli</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000400138/noe-mael-tagne</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000495803/vincenzo-testa</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Noham Hamdaoua</t>
+          <t>Ibrahima Camará</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1295337</v>
+        <v>595012</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -2296,288 +2296,159 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2007-12-16</t>
+          <t>1999-01-25</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2007-01-17</t>
+          <t>2008-05-23</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2000382032</v>
+        <v>2000401946</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>noham-hamdaoua</t>
+          <t>ibrahima-camara</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000382032/noham-hamdaoua</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000401946/ibrahima-camara</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Piergiorgio Bonanno</t>
+          <t>Daniel Mikolajewski</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1190028</v>
+        <v>448567</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Internal transfer: Fiorentina Under 18; date: 01/07/2025</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2007-06-27</t>
+          <t>1999-08-25</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2007-06-26</t>
+          <t>2006-01-24</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>2000333018</v>
+        <v>2000150888</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>piergiorgio-bonanno</t>
+          <t>daniel-mikolajewski</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>ACF Fiorentina</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000333018/piergiorgio-bonanno</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000150888/daniel-mikolajewski</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Raffaele Colella</t>
+          <t>Simone Cinquegrano</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1318329</v>
+        <v>919669</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Napoli Primavera</t>
+          <t>Inter U23</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2006-05-01</t>
+          <t>2004-06-25</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2006-05-04</t>
+          <t>2004-05-25</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>2000266816</v>
+        <v>2000124322</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>raffaele-colella</t>
+          <t>simone-cinquegrano</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>SSC Napoli</t>
+          <t>US Sassuolo</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266816/raffaele-colella</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000124322/simone-cinquegrano</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Riccardo Biguzzi</t>
+          <t>Mattia Brugarello</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1296430</v>
+        <v>898821</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Internal transfer: Cesena Under 18; date: 01/07/2025</t>
+          <t>Juventus Next Gen</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2005-10-28</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2007-02-06</t>
+          <t>2005-10-20</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>2000284347</v>
+        <v>2000098492</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>riccardo-biguzzi</t>
+          <t>mattia-brugarello</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Cesena FC</t>
+          <t>Juventus Next Gen</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284347/riccardo-biguzzi</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Salvatore De Martino</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>1440090</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>New arrival</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>2007-09-24</t>
-        </is>
-      </c>
-      <c r="F48" t="n">
-        <v>2000266709</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>salvatore-de-martino</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>SSC Napoli</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266709/salvatore-de-martino</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Tommaso Reali</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>1311736</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Internal transfer: Frosinone Under 17; date: 01/07/2025</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2008-03-25</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>2008-01-01</t>
-        </is>
-      </c>
-      <c r="F49" t="n">
-        <v>2000495914</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>tommaso-reali</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Frosinone Calcio</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495914/tommaso-reali</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Vincenzo Testa</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>1243102</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Internal transfer: Napoli Under 18; date: 01/07/2025</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>2007-01-01</t>
-        </is>
-      </c>
-      <c r="F50" t="n">
-        <v>2000495803</v>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>vincenzo-testa</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>SSC Napoli</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495803/vincenzo-testa</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000098492/mattia-brugarello</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sots): recupero 31 match cross-club (filtro anno+club per DOB tronche Primavera)
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_dob_mismatch.xlsx
+++ b/data/sots_more_matches_dob_mismatch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -778,15 +778,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Andrea Caucci</t>
+          <t>Andrea Lantignotti</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1051116</v>
+        <v>1296425</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Napoli Primavera</t>
+          <t>Cesena Primavera</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -796,40 +796,40 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2007-06-30</t>
+          <t>2007-05-31</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2000266831</v>
+        <v>2000284355</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>andrea-caucci</t>
+          <t>andrea-lantignotti</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SSC Napoli</t>
+          <t>Cesena FC</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266831/andrea-caucci</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000284355/andrea-lantignotti</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Andrea Lantignotti</t>
+          <t>Bruno Zorzetto</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1296425</v>
+        <v>1182950</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cesena Primavera</t>
+          <t>Frosinone Primavera</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -839,40 +839,40 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2007-05-31</t>
+          <t>2007-12-21</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2000284355</v>
+        <v>2000495913</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>andrea-lantignotti</t>
+          <t>bruno-zorzetto</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Cesena FC</t>
+          <t>Frosinone Calcio</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284355/andrea-lantignotti</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000495913/bruno-zorzetto</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bruno Zorzetto</t>
+          <t>Catello Amendola</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1182950</v>
+        <v>1133143</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Frosinone Primavera</t>
+          <t>Sassuolo Primavera</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -882,208 +882,208 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2007-12-21</t>
+          <t>2007-02-04</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2000495913</v>
+        <v>2000268221</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>bruno-zorzetto</t>
+          <t>catello-amendola</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Frosinone Calcio</t>
+          <t>US Sassuolo</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495913/bruno-zorzetto</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000268221/catello-amendola</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bryant Nieling</t>
+          <t>Diego Tampieri</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>698082</v>
+        <v>1129564</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Modena FC</t>
+          <t>Sassuolo Primavera</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2002-10-31</t>
+          <t>2006-01-25</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2001-11-30</t>
+          <t>2006-01-01</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2000017548</v>
+        <v>2000187279</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>bryant-nieling</t>
+          <t>diego-tampieri</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Modena FC</t>
+          <t>US Sassuolo</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000017548/bryant-nieling</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000187279/diego-tampieri</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Catello Amendola</t>
+          <t>Divine Onyemachi</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1133143</v>
+        <v>1117532</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Lecce Primavera</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2007-08-02</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2007-02-04</t>
+          <t>2006-12-13</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2000268221</v>
+        <v>2000307954</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>catello-amendola</t>
+          <t>divine-onyemachi</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>US Lecce</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268221/catello-amendola</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000307954/divine-onyemachi</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Diego Tampieri</t>
+          <t>Emilio Amadori</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1129564</v>
+        <v>1296435</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Cesena Primavera</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2006-01-25</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2006-01-01</t>
+          <t>2007-01-08</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2000187279</v>
+        <v>2000284319</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>diego-tampieri</t>
+          <t>emilio-amadori</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Cesena FC</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000187279/diego-tampieri</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000284319/emilio-amadori</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Divine Onyemachi</t>
+          <t>Francesco Leone</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1117532</v>
+        <v>1182369</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lecce Primavera</t>
+          <t>Juventus Primavera</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2007-08-02</t>
+          <t>2007-05-03</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2006-12-13</t>
+          <t>2007-05-30</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2000307954</v>
+        <v>2000332032</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>divine-onyemachi</t>
+          <t>francesco-leone</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>US Lecce</t>
+          <t>Juventus FC</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000307954/divine-onyemachi</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000332032/francesco-leone</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Eddy Kouadio</t>
+          <t>Gianmaria Fei</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>957822</v>
+        <v>1317913</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1092,20 +1092,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2006-05-07</t>
+          <t>2007-04-15</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2006-05-03</t>
+          <t>2007-04-17</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2000184141</v>
+        <v>2000403058</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>eddy-kouadio</t>
+          <t>gianmaria-fei</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1115,409 +1115,409 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000184141/eddy-kouadio</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000403058/gianmaria-fei</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Emilio Amadori</t>
+          <t>Giovanni Andrea Cardu</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1296435</v>
+        <v>1253653</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cesena Primavera</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2008-05-11</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2007-01-08</t>
+          <t>2008-05-19</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2000284319</v>
+        <v>2000461316</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>emilio-amadori</t>
+          <t>giovanni-andrea-cardu</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Cesena FC</t>
+          <t>Cagliari Calcio</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284319/emilio-amadori</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000461316/giovanni-andrea-cardu</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Francesco Leone</t>
+          <t>Isaac Enoghama</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1182369</v>
+        <v>1075420</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Juventus Primavera</t>
+          <t>Genoa Primavera</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2007-05-03</t>
+          <t>2007-09-10</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2007-05-30</t>
+          <t>2007-08-10</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2000332032</v>
+        <v>2000266435</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>francesco-leone</t>
+          <t>isaac-enoghama</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Juventus FC</t>
+          <t>Genoa CFC</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000332032/francesco-leone</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000266435/isaac-enoghama</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gianmaria Fei</t>
+          <t>Jack Nunn</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1317913</v>
+        <v>1292591</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fiorentina Primavera</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2007-04-15</t>
+          <t>2006-07-07</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2007-04-17</t>
+          <t>2006-07-08</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2000403058</v>
+        <v>2000389422</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>gianmaria-fei</t>
+          <t>jack-nunn</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ACF Fiorentina</t>
+          <t>Cagliari Calcio</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000403058/gianmaria-fei</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000389422/jack-nunn</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Giovanni Andrea Cardu</t>
+          <t>Lorenzo Nyarko</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1253653</v>
+        <v>1168024</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cagliari Primavera</t>
+          <t>Sassuolo Primavera</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2008-05-11</t>
+          <t>2007-10-20</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2008-05-19</t>
+          <t>2007-08-20</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2000461316</v>
+        <v>2000268210</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>giovanni-andrea-cardu</t>
+          <t>lorenzo-nyarko</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>US Sassuolo</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000461316/giovanni-andrea-cardu</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000268210/lorenzo-nyarko</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ioan Vermeșan</t>
+          <t>Lorenzo Pio Marino</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>928037</v>
+        <v>1100015</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hellas Verona Primavera</t>
+          <t>Cremonese Primavera</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2006-10-18</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2006-10-15</t>
+          <t>2007-01-03</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2000157324</v>
+        <v>2000261855</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ioan-vermesan</t>
+          <t>lorenzo-pio-marino</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Hellas Verona</t>
+          <t>US Cremonese</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000157324/ioan-vermesan</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000261855/lorenzo-pio-marino</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Isaac Enoghama</t>
+          <t>Luca Gobbo</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1075420</v>
+        <v>1183953</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Genoa Primavera</t>
+          <t>Atalanta Primavera</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2007-09-10</t>
+          <t>2006-04-05</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2007-08-10</t>
+          <t>2006-04-07</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2000266435</v>
+        <v>2000333546</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>isaac-enoghama</t>
+          <t>luca-gobbo</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Genoa CFC</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266435/isaac-enoghama</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000333546/luca-gobbo</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jack Nunn</t>
+          <t>Ludovico Varali</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1292591</v>
+        <v>1388316</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Cagliari Primavera</t>
+          <t>Parma Primavera</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2006-07-07</t>
+          <t>2009-01-17</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2006-07-08</t>
+          <t>2009-01-06</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2000389422</v>
+        <v>2000491914</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>jack-nunn</t>
+          <t>ludovico-varali</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000389422/jack-nunn</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000491914/ludovico-varali</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Joseph Liteta</t>
+          <t>Mark Topollaj</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1134304</v>
+        <v>949340</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Cagliari Primavera</t>
+          <t>Hellas Verona Primavera</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2006-02-22</t>
+          <t>2007-09-25</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2006-01-22</t>
+          <t>2007-08-25</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2000241198</v>
+        <v>2000269202</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>joseph-liteta</t>
+          <t>mark-topollaj</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Hellas Verona</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000241198/joseph-liteta</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000269202/mark-topollaj</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Lorenzo Nyarko</t>
+          <t>Márton Prettenhoffer</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1168024</v>
+        <v>1060896</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2007-10-20</t>
+          <t>2008-03-10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2007-08-20</t>
+          <t>2008-03-17</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2000268210</v>
+        <v>2000394155</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>lorenzo-nyarko</t>
+          <t>marton-prettenhoffer</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Cagliari Calcio</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268210/lorenzo-nyarko</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000394155/marton-prettenhoffer</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Lorenzo Pio Marino</t>
+          <t>Mattia Aliprandi</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1100015</v>
+        <v>1170819</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cremonese Primavera</t>
+          <t>Atalanta Primavera</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1527,341 +1527,341 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2007-01-03</t>
+          <t>2007-01-04</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2000261855</v>
+        <v>2000330730</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>lorenzo-pio-marino</t>
+          <t>mattia-aliprandi</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>US Cremonese</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000261855/lorenzo-pio-marino</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000330730/mattia-aliprandi</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Luca Gobbo</t>
+          <t>Noe Mael Tagne</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1183953</v>
+        <v>1310290</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Atalanta Primavera</t>
+          <t>Hellas Verona Primavera</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2006-04-05</t>
+          <t>2008-08-08</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2006-04-07</t>
+          <t>2008-08-11</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2000333546</v>
+        <v>2000400138</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>luca-gobbo</t>
+          <t>noe-mael-tagne</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Atalanta BC</t>
+          <t>Hellas Verona</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000333546/luca-gobbo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000400138/noe-mael-tagne</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ludovico Varali</t>
+          <t>Noham Hamdaoua</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1388316</v>
+        <v>1295337</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Parma Primavera</t>
+          <t>Cagliari Primavera</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2009-01-17</t>
+          <t>2007-12-16</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2009-01-06</t>
+          <t>2007-01-17</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2000491914</v>
+        <v>2000382032</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>ludovico-varali</t>
+          <t>noham-hamdaoua</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Cagliari Calcio</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000491914/ludovico-varali</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000382032/noham-hamdaoua</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Marco Tiozzo</t>
+          <t>Piergiorgio Bonanno</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1234457</v>
+        <v>1190028</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Juventus Primavera</t>
+          <t>Fiorentina Primavera</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2008-10-07</t>
+          <t>2007-06-27</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2008-07-10</t>
+          <t>2007-06-26</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2000386592</v>
+        <v>2000333018</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>marco-tiozzo-pagio</t>
+          <t>piergiorgio-bonanno</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Juventus FC</t>
+          <t>ACF Fiorentina</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000386592/marco-tiozzo-pagio</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000333018/piergiorgio-bonanno</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Mariano Troilo</t>
+          <t>Raffaele Colella</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1159864</v>
+        <v>1318329</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2003-06-28</t>
+          <t>2006-05-01</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2003-06-22</t>
+          <t>2006-05-04</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2000200406</v>
+        <v>2000266816</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>mariano-troilo</t>
+          <t>raffaele-colella</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>SSC Napoli</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000200406/mariano-troilo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000266816/raffaele-colella</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mark Topollaj</t>
+          <t>Riccardo Biguzzi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>949340</v>
+        <v>1296430</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Hellas Verona Primavera</t>
+          <t>Cesena Primavera</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2007-09-25</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2007-08-25</t>
+          <t>2007-02-06</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>2000269202</v>
+        <v>2000284347</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>mark-topollaj</t>
+          <t>riccardo-biguzzi</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Hellas Verona</t>
+          <t>Cesena FC</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000269202/mark-topollaj</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000284347/riccardo-biguzzi</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Marko Farji</t>
+          <t>Salvatore De Martino</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>663153</v>
+        <v>1440090</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Venezia FC</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2004-03-16</t>
+          <t>2007 (~ 19</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2004-03-26</t>
+          <t>2007-09-24</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2000065330</v>
+        <v>2000266709</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>marko-farji</t>
+          <t>salvatore-de-martino</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Venezia FC</t>
+          <t>SSC Napoli</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000065330/marko-farji</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000266709/salvatore-de-martino</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Márton Prettenhoffer</t>
+          <t>Tommaso Reali</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1060896</v>
+        <v>1311736</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Cagliari Primavera</t>
+          <t>Frosinone Primavera</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2008-03-10</t>
+          <t>2008-03-25</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2008-03-17</t>
+          <t>2008-01-01</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2000394155</v>
+        <v>2000495914</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>marton-prettenhoffer</t>
+          <t>tommaso-reali</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Frosinone Calcio</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000394155/marton-prettenhoffer</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000495914/tommaso-reali</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mattia Aliprandi</t>
+          <t>Vincenzo Testa</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1170819</v>
+        <v>1243102</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Atalanta Primavera</t>
+          <t>Napoli Primavera</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1871,584 +1871,111 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2007-01-04</t>
+          <t>2007-01-01</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>2000330730</v>
+        <v>2000495803</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>mattia-aliprandi</t>
+          <t>vincenzo-testa</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Atalanta BC</t>
+          <t>SSC Napoli</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000330730/mattia-aliprandi</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000495803/vincenzo-testa</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Michael Zeppieri</t>
+          <t>Ibrahima Camará</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1084276</v>
+        <v>595012</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Torino Primavera</t>
+          <t>Radomiak</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2006-06-01</t>
+          <t>1999-01-25</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2006-09-23</t>
+          <t>2008-05-23</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2000269983</v>
+        <v>2000401946</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>michael-zeppieri</t>
+          <t>ibrahima-camara</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Torino FC</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000269983/michael-zeppieri</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000401946/ibrahima-camara</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Noe Mael Tagne</t>
+          <t>Daniel Mikolajewski</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1310290</v>
+        <v>448567</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hellas Verona Primavera</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2008-08-08</t>
+          <t>1999-08-25</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2008-08-11</t>
+          <t>2006-01-24</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2000400138</v>
+        <v>2000150888</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>noe-mael-tagne</t>
+          <t>daniel-mikolajewski</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Hellas Verona</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000400138/noe-mael-tagne</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Noham Hamdaoua</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1295337</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Cagliari Primavera</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2007-12-16</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2007-01-17</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>2000382032</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>noham-hamdaoua</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Cagliari Calcio</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000382032/noham-hamdaoua</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Piergiorgio Bonanno</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1190028</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Fiorentina Primavera</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>2007-06-27</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>2007-06-26</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>2000333018</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>piergiorgio-bonanno</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>ACF Fiorentina</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000333018/piergiorgio-bonanno</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Raffaele Colella</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1318329</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Napoli Primavera</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>2006-05-01</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2006-05-04</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>2000266816</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>raffaele-colella</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>SSC Napoli</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266816/raffaele-colella</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Riccardo Biguzzi</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1296430</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Cesena Primavera</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2007-02-06</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>2000284347</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>riccardo-biguzzi</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Cesena FC</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284347/riccardo-biguzzi</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Salvatore De Martino</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1440090</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Napoli Primavera</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2007-09-24</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>2000266709</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>salvatore-de-martino</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>SSC Napoli</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266709/salvatore-de-martino</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Tommaso Reali</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1311736</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Frosinone Primavera</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2008-03-25</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2008-01-01</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>2000495914</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>tommaso-reali</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Frosinone Calcio</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495914/tommaso-reali</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Vincenzo Testa</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1243102</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Napoli Primavera</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>2007-01-01</t>
-        </is>
-      </c>
-      <c r="F43" t="n">
-        <v>2000495803</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>vincenzo-testa</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>SSC Napoli</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495803/vincenzo-testa</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Ibrahima Camará</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>595012</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>New arrival</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>1999-01-25</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>2008-05-23</t>
-        </is>
-      </c>
-      <c r="F44" t="n">
-        <v>2000401946</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>ibrahima-camara</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Atalanta BC</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000401946/ibrahima-camara</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Daniel Mikolajewski</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>448567</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Wieczysta Krakow</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>1999-08-25</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>2006-01-24</t>
-        </is>
-      </c>
-      <c r="F45" t="n">
-        <v>2000150888</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>daniel-mikolajewski</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Parma Calcio 1913</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
           <t>https://sortitoutsi.net/football-manager-2026/person/2000150888/daniel-mikolajewski</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Simone Cinquegrano</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>919669</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Inter U23</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>2004-06-25</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>2004-05-25</t>
-        </is>
-      </c>
-      <c r="F46" t="n">
-        <v>2000124322</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>simone-cinquegrano</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>US Sassuolo</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000124322/simone-cinquegrano</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Mattia Brugarello</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>898821</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Juventus Next Gen</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2005-10-28</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>2005-10-20</t>
-        </is>
-      </c>
-      <c r="F47" t="n">
-        <v>2000098492</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>mattia-brugarello</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Juventus Next Gen</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000098492/mattia-brugarello</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sots): aggiunte PL1/PL2 (Ekstraklasa/I Liga) — recupero 784 foto polacchi via harvest cross-club
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_dob_mismatch.xlsx
+++ b/data/sots_more_matches_dob_mismatch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -477,1505 +477,946 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Abubacar Ceesay</t>
+          <t>Divine Onyemachi</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1462448</v>
+        <v>1117532</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Frosinone Primavera</t>
+          <t>Lecce Primavera</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2007-08-02</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2007-10-19</t>
+          <t>2006-12-13</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2000506803</v>
+        <v>2000307954</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>abubacar-ceesay</t>
+          <t>divine-onyemachi</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Frosinone Calcio</t>
+          <t>US Lecce</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000506803/abubacar-ceesay</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000307954/divine-onyemachi</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Adam Hasani</t>
+          <t>Kuba Nawrocki</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1246891</v>
+        <v>1426749</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Napoli Primavera</t>
+          <t>Internal transfer: Widzew Lodz II; date: 15/07/2025</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2008-09-05</t>
+          <t>2007-04-03</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2008-08-05</t>
+          <t>2007-04-02</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2000390952</v>
+        <v>2000438522</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>adam-hasani</t>
+          <t>kuba-nawrocki</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SSC Napoli</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000390952/adam-hasani</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000438522/kuba-nawrocki</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alessandro Bagnaschi</t>
+          <t>Borislav Rupanov</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1060357</v>
+        <v>1006467</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Monza Primavera</t>
+          <t>Levski Sofia</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2006 (~ 20</t>
+          <t>2004-11-30</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2006-06-09</t>
+          <t>2004-08-01</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2000241770</v>
+        <v>2000183319</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>alessandro-bagnaschi</t>
+          <t>borislav-rupanov</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>AC Monza</t>
+          <t>Górnik Zabrze</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000241770/alessandro-bagnaschi</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000183319/borislav-rupanov</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alessio Sibilano</t>
+          <t>Viktor Popov</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1168030</v>
+        <v>634145</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2000-03-05</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2007-07-06</t>
+          <t>2000-03-06</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2000268216</v>
+        <v>31040477</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>alessio-sibilano</t>
+          <t>viktor-popov</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268216/alessio-sibilano</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/31040477/viktor-popov</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alfonso De Luca</t>
+          <t>Nono</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1077899</v>
+        <v>152776</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Napoli Primavera</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2006-09-19</t>
+          <t>1991-05-28</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2006-06-19</t>
+          <t>1991-06-28</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2000242306</v>
+        <v>67144727</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>alfonso-de-luca</t>
+          <t>nono</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SSC Napoli</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000242306/alfonso-de-luca</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/67144727/nono</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Alfonso De Luca</t>
+          <t>Fabian Hiszpański</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1077899</v>
+        <v>194139</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Napoli Primavera</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2006-09-19</t>
+          <t>1993-10-26</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1997-07-14</t>
+          <t>1993-10-28</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2000427316</v>
+        <v>96027813</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>alfonso-de-luca</t>
+          <t>fabian-hiszpanski</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>US Avellino 1912</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000427316/alfonso-de-luca</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/96027813/fabian-hiszpanski</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Andrea Campani</t>
+          <t>Oskar Markiewicz</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1044819</v>
+        <v>1520380</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Internal transfer: Radomiak Radom II; date: 27/02/2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>1999-12-10</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2007-04-03</t>
+          <t>1999-12-06</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2000268200</v>
+        <v>2000438722</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>andrea-campani</t>
+          <t>oskar-markiewicz</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268200/andrea-campani</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000438722/oskar-markiewicz</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Andrea Lantignotti</t>
+          <t>Ibrahima Camará</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1296425</v>
+        <v>595012</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cesena Primavera</t>
+          <t>Radomiak</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>1999-01-25</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2007-05-31</t>
+          <t>2008-05-23</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2000284355</v>
+        <v>2000401946</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>andrea-lantignotti</t>
+          <t>ibrahima-camara</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Cesena FC</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284355/andrea-lantignotti</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000401946/ibrahima-camara</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bruno Zorzetto</t>
+          <t>Jakub Grelich</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1182950</v>
+        <v>1510054</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Frosinone Primavera</t>
+          <t>Internal transfer: Piast Gliwice II; date: 02/02/2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2008-05-25</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2007-12-21</t>
+          <t>2008-04-15</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2000495913</v>
+        <v>2000529507</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>bruno-zorzetto</t>
+          <t>jakub-grelich</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Frosinone Calcio</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495913/bruno-zorzetto</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000529507/jakub-grelich</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Catello Amendola</t>
+          <t>Szczepan Mucha</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1133143</v>
+        <v>726397</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Rekord Bielsko-Biala</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2004-02-29</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2007-02-04</t>
+          <t>2004-04-29</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2000268221</v>
+        <v>2000009023</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>catello-amendola</t>
+          <t>szczepan-mucha</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268221/catello-amendola</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000009023/szczepan-mucha</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Diego Tampieri</t>
+          <t>Sergio Guerrero</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1129564</v>
+        <v>606570</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2006-01-25</t>
+          <t>1999-04-10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2006-01-01</t>
+          <t>1999-01-13</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2000187279</v>
+        <v>67262228</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>diego-tampieri</t>
+          <t>sergio-guerrero</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Bruk-Bet Termalica Nieciecza</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000187279/diego-tampieri</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/67262228/sergio-guerrero</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Divine Onyemachi</t>
+          <t>Daniel Mikolajewski</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1117532</v>
+        <v>448567</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Lecce Primavera</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2007-08-02</t>
+          <t>1999-08-25</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2006-12-13</t>
+          <t>2006-01-24</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2000307954</v>
+        <v>2000150888</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>divine-onyemachi</t>
+          <t>daniel-mikolajewski</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>US Lecce</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000307954/divine-onyemachi</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000150888/daniel-mikolajewski</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Emilio Amadori</t>
+          <t>Dave Gnaase</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1296435</v>
+        <v>286593</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cesena Primavera</t>
+          <t>Pol. Warsaw</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>1996-12-14</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2007-01-08</t>
+          <t>1996-12-26</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2000284319</v>
+        <v>92074814</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>emilio-amadori</t>
+          <t>dave-gnaase</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Cesena FC</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284319/emilio-amadori</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/92074814/dave-gnaase</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Francesco Leone</t>
+          <t>Maksymilian Dziuba</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1182369</v>
+        <v>930125</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Juventus Primavera</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2007-05-03</t>
+          <t>2005-07-01</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2007-05-30</t>
+          <t>2005-05-01</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2000332032</v>
+        <v>2000133218</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>francesco-leone</t>
+          <t>maksymilian-dziuba</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Juventus FC</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000332032/francesco-leone</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000133218/maksymilian-dziuba</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gianmaria Fei</t>
+          <t>Filip Sonntag</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1317913</v>
+        <v>1268625</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fiorentina Primavera</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2007-04-15</t>
+          <t>2008-06-09</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2007-04-17</t>
+          <t>2008-06-08</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2000403058</v>
+        <v>2000444481</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gianmaria-fei</t>
+          <t>filip-sonntag</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ACF Fiorentina</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000403058/gianmaria-fei</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000444481/filip-sonntag</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Giovanni Andrea Cardu</t>
+          <t>Mateusz Lewandowski</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1253653</v>
+        <v>438351</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cagliari Primavera</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2008-05-11</t>
+          <t>1999-03-04</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2008-05-19</t>
+          <t>1993-03-18</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2000461316</v>
+        <v>96017250</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>giovanni-andrea-cardu</t>
+          <t>mateusz-lewandowski</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000461316/giovanni-andrea-cardu</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/96017250/mateusz-lewandowski</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Isaac Enoghama</t>
+          <t>Jakub Lis</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1075420</v>
+        <v>1165401</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Genoa Primavera</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2007-09-10</t>
+          <t>2004-10-14</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2007-08-10</t>
+          <t>2002-01-14</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2000266435</v>
+        <v>2000037232</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>isaac-enoghama</t>
+          <t>jakub-lis</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Genoa CFC</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266435/isaac-enoghama</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000037232/jakub-lis</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Jack Nunn</t>
+          <t>Mateusz Ozimek</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1292591</v>
+        <v>549313</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cagliari Primavera</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2006-07-07</t>
+          <t>2000-06-21</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2006-07-08</t>
+          <t>1995-12-18</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2000389422</v>
+        <v>2000045929</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>jack-nunn</t>
+          <t>mateusz-ozimek</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Cagliari Calcio</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000389422/jack-nunn</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000045929/mateusz-ozimek</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lorenzo Nyarko</t>
+          <t>Jakub Szymański</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1168024</v>
+        <v>798319</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sassuolo Primavera</t>
+          <t>Polonia Bytom</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2007-10-20</t>
+          <t>2002-07-05</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2007-08-20</t>
+          <t>2000-08-30</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2000268210</v>
+        <v>96125541</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>lorenzo-nyarko</t>
+          <t>jakub-szymanski</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>US Sassuolo</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000268210/lorenzo-nyarko</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/96125541/jakub-szymanski</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lorenzo Pio Marino</t>
+          <t>Nico Adamczyk</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1100015</v>
+        <v>884808</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cremonese Primavera</t>
+          <t>GKS Tychy</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2007 (~ 19</t>
+          <t>2006-01-25</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2007-01-03</t>
+          <t>2006-01-15</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2000261855</v>
+        <v>2000182173</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>lorenzo-pio-marino</t>
+          <t>nico-adamczyk</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>US Cremonese</t>
+          <t>GKS Tychy</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000261855/lorenzo-pio-marino</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000182173/nico-adamczyk</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Luca Gobbo</t>
+          <t>Jan Stępniak</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1183953</v>
+        <v>1516608</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Atalanta Primavera</t>
+          <t>Internal transfer: Gornik Leczna II; date: 18/02/2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2006-04-05</t>
+          <t>2009-02-01</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2006-04-07</t>
+          <t>2009-01-01</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2000333546</v>
+        <v>2000525900</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>luca-gobbo</t>
+          <t>jan-stepniak</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Atalanta BC</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000333546/luca-gobbo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000525900/jan-stepniak</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ludovico Varali</t>
+          <t>Sebastian Szczytniewski</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1388316</v>
+        <v>805499</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Parma Primavera</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2009-01-17</t>
+          <t>2003-03-19</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2009-01-06</t>
+          <t>2003-03-13</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2000491914</v>
+        <v>2000047883</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ludovico-varali</t>
+          <t>sebastian-szczytniewski</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000491914/ludovico-varali</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Mark Topollaj</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>949340</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Hellas Verona Primavera</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2007-09-25</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>2007-08-25</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>2000269202</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>mark-topollaj</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Hellas Verona</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000269202/mark-topollaj</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Márton Prettenhoffer</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1060896</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Cagliari Primavera</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2008-03-10</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2008-03-17</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>2000394155</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>marton-prettenhoffer</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Cagliari Calcio</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000394155/marton-prettenhoffer</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Mattia Aliprandi</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1170819</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Atalanta Primavera</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2007-01-04</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>2000330730</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>mattia-aliprandi</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Atalanta BC</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000330730/mattia-aliprandi</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Noe Mael Tagne</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>1310290</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Hellas Verona Primavera</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2008-08-08</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2008-08-11</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>2000400138</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>noe-mael-tagne</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Hellas Verona</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000400138/noe-mael-tagne</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Noham Hamdaoua</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1295337</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Cagliari Primavera</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>2007-12-16</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2007-01-17</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>2000382032</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>noham-hamdaoua</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Cagliari Calcio</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000382032/noham-hamdaoua</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Piergiorgio Bonanno</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1190028</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Fiorentina Primavera</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>2007-06-27</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2007-06-26</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>2000333018</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>piergiorgio-bonanno</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>ACF Fiorentina</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000333018/piergiorgio-bonanno</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Raffaele Colella</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1318329</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Napoli Primavera</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>2006-05-01</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2006-05-04</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>2000266816</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>raffaele-colella</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>SSC Napoli</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266816/raffaele-colella</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Riccardo Biguzzi</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1296430</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Cesena Primavera</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2007-02-06</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>2000284347</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>riccardo-biguzzi</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Cesena FC</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000284347/riccardo-biguzzi</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Salvatore De Martino</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1440090</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Napoli Primavera</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2007-09-24</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>2000266709</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>salvatore-de-martino</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>SSC Napoli</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266709/salvatore-de-martino</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Tommaso Reali</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1311736</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Frosinone Primavera</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>2008-03-25</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>2008-01-01</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>2000495914</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>tommaso-reali</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Frosinone Calcio</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495914/tommaso-reali</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Vincenzo Testa</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>1243102</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Napoli Primavera</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>2007 (~ 19</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2007-01-01</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>2000495803</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>vincenzo-testa</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>SSC Napoli</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000495803/vincenzo-testa</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Ibrahima Camará</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>595012</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Radomiak</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>1999-01-25</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2008-05-23</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>2000401946</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>ibrahima-camara</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Atalanta BC</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000401946/ibrahima-camara</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Daniel Mikolajewski</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>448567</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Wieczysta Krakow</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>1999-08-25</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2006-01-24</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>2000150888</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>daniel-mikolajewski</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Parma Calcio 1913</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000150888/daniel-mikolajewski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000047883/sebastian-szczytniewski</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sots): +141 auto via fix slugify Ł→l + 4 override manuali — foto SOTS 95.4% (era 90.3%, era 62% inizio giornata)
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_dob_mismatch.xlsx
+++ b/data/sots_more_matches_dob_mismatch.xlsx
@@ -778,76 +778,76 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ibrahima Camará</t>
+          <t>Jakub Grelich</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>595012</v>
+        <v>1510054</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Radomiak</t>
+          <t>Internal transfer: Piast Gliwice II; date: 02/02/2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1999-01-25</t>
+          <t>2008-05-25</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2008-05-23</t>
+          <t>2008-04-15</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2000401946</v>
+        <v>2000529507</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>ibrahima-camara</t>
+          <t>jakub-grelich</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Atalanta BC</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000401946/ibrahima-camara</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000529507/jakub-grelich</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jakub Grelich</t>
+          <t>Szczepan Mucha</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1510054</v>
+        <v>726397</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Internal transfer: Piast Gliwice II; date: 02/02/2026</t>
+          <t>Rekord Bielsko-Biala</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2008-05-25</t>
+          <t>2004-02-29</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2008-04-15</t>
+          <t>2004-04-29</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2000529507</v>
+        <v>2000009023</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>jakub-grelich</t>
+          <t>szczepan-mucha</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -857,169 +857,169 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000529507/jakub-grelich</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000009023/szczepan-mucha</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Szczepan Mucha</t>
+          <t>Sergio Guerrero</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>726397</v>
+        <v>606570</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Rekord Bielsko-Biala</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2004-02-29</t>
+          <t>1999-04-10</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2004-04-29</t>
+          <t>1999-01-13</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2000009023</v>
+        <v>67262228</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>szczepan-mucha</t>
+          <t>sergio-guerrero</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Bruk-Bet Termalica Nieciecza</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000009023/szczepan-mucha</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/67262228/sergio-guerrero</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sergio Guerrero</t>
+          <t>Daniel Mikolajewski</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>606570</v>
+        <v>448567</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Nieciecza</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1999-04-10</t>
+          <t>1999-08-25</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1999-01-13</t>
+          <t>2006-01-24</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>67262228</v>
+        <v>2000150888</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>sergio-guerrero</t>
+          <t>daniel-mikolajewski</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Bruk-Bet Termalica Nieciecza</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/67262228/sergio-guerrero</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000150888/daniel-mikolajewski</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Daniel Mikolajewski</t>
+          <t>Dave Gnaase</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>448567</v>
+        <v>286593</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>Pol. Warsaw</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1999-08-25</t>
+          <t>1996-12-14</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2006-01-24</t>
+          <t>1996-12-26</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2000150888</v>
+        <v>92074814</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>daniel-mikolajewski</t>
+          <t>dave-gnaase</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000150888/daniel-mikolajewski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/92074814/dave-gnaase</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dave Gnaase</t>
+          <t>Kacper Ziółkowski</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>286593</v>
+        <v>1521095</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pol. Warsaw</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1996-12-14</t>
+          <t>2009-09-26</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1996-12-26</t>
+          <t>2009-01-01</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>92074814</v>
+        <v>2000525889</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>dave-gnaase</t>
+          <t>kacper-ziolkowski</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/92074814/dave-gnaase</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000525889/kacper-ziolkowski</t>
         </is>
       </c>
     </row>
@@ -1122,301 +1122,301 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mateusz Lewandowski</t>
+          <t>Jakub Lis</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>438351</v>
+        <v>1165401</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1999-03-04</t>
+          <t>2004-10-14</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1993-03-18</t>
+          <t>2002-01-14</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>96017250</v>
+        <v>2000037232</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>mateusz-lewandowski</t>
+          <t>jakub-lis</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96017250/mateusz-lewandowski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000037232/jakub-lis</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Jakub Lis</t>
+          <t>Nico Adamczyk</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1165401</v>
+        <v>884808</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>GKS Tychy</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2004-10-14</t>
+          <t>2006-01-25</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2002-01-14</t>
+          <t>2006-01-15</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2000037232</v>
+        <v>2000182173</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>jakub-lis</t>
+          <t>nico-adamczyk</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>GKS Tychy</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000037232/jakub-lis</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000182173/nico-adamczyk</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mateusz Ozimek</t>
+          <t>Kacper Przybyłko</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>549313</v>
+        <v>952379</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>P. Niepolomice</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2000-06-21</t>
+          <t>2005-02-05</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1995-12-18</t>
+          <t>1993-03-25</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2000045929</v>
+        <v>91109529</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>mateusz-ozimek</t>
+          <t>kacper-przybylko</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000045929/mateusz-ozimek</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/91109529/kacper-przybylko</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jakub Szymański</t>
+          <t>Jan Stępniak</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>798319</v>
+        <v>1516608</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Polonia Bytom</t>
+          <t>Internal transfer: Gornik Leczna II; date: 18/02/2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2002-07-05</t>
+          <t>2009-02-01</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2000-08-30</t>
+          <t>2009-01-01</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>96125541</v>
+        <v>2000525900</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>jakub-szymanski</t>
+          <t>jan-stepniak</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96125541/jakub-szymanski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000525900/jan-stepniak</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nico Adamczyk</t>
+          <t>Krystian Kołodziejczak</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>884808</v>
+        <v>1516583</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GKS Tychy</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2006-01-25</t>
+          <t>2009-09-04</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2006-01-15</t>
+          <t>2009-01-01</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2000182173</v>
+        <v>2000525898</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nico-adamczyk</t>
+          <t>krystian-kolodziejczak</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>GKS Tychy</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000182173/nico-adamczyk</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000525898/krystian-kolodziejczak</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jan Stępniak</t>
+          <t>Sebastian Szczytniewski</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1516608</v>
+        <v>805499</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Internal transfer: Gornik Leczna II; date: 18/02/2026</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2009-02-01</t>
+          <t>2003-03-19</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2009-01-01</t>
+          <t>2003-03-13</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2000525900</v>
+        <v>2000047883</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>jan-stepniak</t>
+          <t>sebastian-szczytniewski</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Gornik Leczna</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000525900/jan-stepniak</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000047883/sebastian-szczytniewski</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sebastian Szczytniewski</t>
+          <t>Przemysław Misiak</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>805499</v>
+        <v>900848</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Gornik Leczna</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2003-03-19</t>
+          <t>2003-08-29</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2003-03-13</t>
+          <t>2003-08-23</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2000047883</v>
+        <v>96161668</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>sebastian-szczytniewski</t>
+          <t>przemyslaw-misiak</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000047883/sebastian-szczytniewski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/96161668/przemyslaw-misiak</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SOTS more matches: +30 confermati DOB (Gubbio 23/23 + altri 7)
Eseguito find_more_sots_matches.py + apply_more_matches.py sul pool
unmatched (55 player senza sortitoutsi_person_id):
- 30 confermati con DOB verificata, 27 DOB mismatch (skippati)
- Tutti i 23 player AS Gubbio 1910 ora hanno sortitoutsi_person_id +
  sortitoutsi_face_local_lookup → foto SOTS visibili nel frontend
- Altri 7 match in vari club (Roma, Bologna, Fiorentina, Sassuolo,
  Verona, Como, Napoli, Juve, Entella, Spezia, Pineto): nuovi
  trasferimenti / loan / Primavera che non erano stati matchati nel
  giro precedente.
- 30 nuove foto face_*.png scaricate nel CDN locale.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_dob_mismatch.xlsx
+++ b/data/sots_more_matches_dob_mismatch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -692,119 +692,119 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fabian Hiszpański</t>
+          <t>Oskar Markiewicz</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>194139</v>
+        <v>1520380</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Internal transfer: Radomiak Radom II; date: 27/02/2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1993-10-26</t>
+          <t>1999-12-10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1993-10-28</t>
+          <t>1999-12-06</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>96027813</v>
+        <v>2000438722</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>fabian-hiszpanski</t>
+          <t>oskar-markiewicz</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96027813/fabian-hiszpanski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000438722/oskar-markiewicz</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oskar Markiewicz</t>
+          <t>Jakub Grelich</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1520380</v>
+        <v>1510054</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Internal transfer: Radomiak Radom II; date: 27/02/2026</t>
+          <t>Internal transfer: Piast Gliwice II; date: 02/02/2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1999-12-10</t>
+          <t>2008-05-25</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1999-12-06</t>
+          <t>2008-04-15</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2000438722</v>
+        <v>2000529507</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>oskar-markiewicz</t>
+          <t>jakub-grelich</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000438722/oskar-markiewicz</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000529507/jakub-grelich</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jakub Grelich</t>
+          <t>Szczepan Mucha</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1510054</v>
+        <v>726397</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Internal transfer: Piast Gliwice II; date: 02/02/2026</t>
+          <t>Rekord Bielsko-Biala</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2008-05-25</t>
+          <t>2004-02-29</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2008-04-15</t>
+          <t>2004-04-29</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2000529507</v>
+        <v>2000009023</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>jakub-grelich</t>
+          <t>szczepan-mucha</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -814,169 +814,169 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000529507/jakub-grelich</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000009023/szczepan-mucha</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Szczepan Mucha</t>
+          <t>Sergio Guerrero</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>726397</v>
+        <v>606570</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Rekord Bielsko-Biala</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2004-02-29</t>
+          <t>1999-04-10</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2004-04-29</t>
+          <t>1999-01-13</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2000009023</v>
+        <v>67262228</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>szczepan-mucha</t>
+          <t>sergio-guerrero</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Bruk-Bet Termalica Nieciecza</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000009023/szczepan-mucha</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/67262228/sergio-guerrero</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sergio Guerrero</t>
+          <t>Daniel Mikolajewski</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>606570</v>
+        <v>448567</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nieciecza</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1999-04-10</t>
+          <t>1999-08-25</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1999-01-13</t>
+          <t>2006-01-24</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>67262228</v>
+        <v>2000150888</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>sergio-guerrero</t>
+          <t>daniel-mikolajewski</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Bruk-Bet Termalica Nieciecza</t>
+          <t>Parma Calcio 1913</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/67262228/sergio-guerrero</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000150888/daniel-mikolajewski</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Daniel Mikolajewski</t>
+          <t>Dave Gnaase</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>448567</v>
+        <v>286593</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>Pol. Warsaw</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1999-08-25</t>
+          <t>1996-12-14</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2006-01-24</t>
+          <t>1996-12-26</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2000150888</v>
+        <v>92074814</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>daniel-mikolajewski</t>
+          <t>dave-gnaase</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Parma Calcio 1913</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000150888/daniel-mikolajewski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/92074814/dave-gnaase</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dave Gnaase</t>
+          <t>Kacper Ziółkowski</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>286593</v>
+        <v>1521095</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pol. Warsaw</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1996-12-14</t>
+          <t>2009-09-26</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1996-12-26</t>
+          <t>2009-01-01</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>92074814</v>
+        <v>2000525889</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>dave-gnaase</t>
+          <t>kacper-ziolkowski</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -986,437 +986,652 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/92074814/dave-gnaase</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000525889/kacper-ziolkowski</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kacper Ziółkowski</t>
+          <t>Maksymilian Dziuba</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1521095</v>
+        <v>930125</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2009-09-26</t>
+          <t>2005-07-01</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2009-01-01</t>
+          <t>2005-05-01</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2000525889</v>
+        <v>2000133218</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>kacper-ziolkowski</t>
+          <t>maksymilian-dziuba</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000525889/kacper-ziolkowski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000133218/maksymilian-dziuba</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Maksymilian Dziuba</t>
+          <t>Filip Sonntag</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>930125</v>
+        <v>1268625</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Slask Wroclaw</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2005-07-01</t>
+          <t>2008-06-09</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2005-05-01</t>
+          <t>2008-06-08</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2000133218</v>
+        <v>2000444481</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>maksymilian-dziuba</t>
+          <t>filip-sonntag</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000133218/maksymilian-dziuba</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000444481/filip-sonntag</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Filip Sonntag</t>
+          <t>Jakub Lis</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1268625</v>
+        <v>1165401</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2008-06-09</t>
+          <t>2004-10-14</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2008-06-08</t>
+          <t>2002-01-14</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2000444481</v>
+        <v>2000037232</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>filip-sonntag</t>
+          <t>jakub-lis</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000444481/filip-sonntag</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000037232/jakub-lis</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jakub Lis</t>
+          <t>Nico Adamczyk</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1165401</v>
+        <v>884808</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>GKS Tychy</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2004-10-14</t>
+          <t>2006-01-25</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2002-01-14</t>
+          <t>2006-01-15</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2000037232</v>
+        <v>2000182173</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>jakub-lis</t>
+          <t>nico-adamczyk</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>GKS Tychy</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000037232/jakub-lis</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000182173/nico-adamczyk</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nico Adamczyk</t>
+          <t>Jan Stępniak</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>884808</v>
+        <v>1516608</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GKS Tychy</t>
+          <t>Internal transfer: Gornik Leczna II; date: 18/02/2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2006-01-25</t>
+          <t>2009-02-01</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2006-01-15</t>
+          <t>2009-01-01</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2000182173</v>
+        <v>2000525900</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nico-adamczyk</t>
+          <t>jan-stepniak</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>GKS Tychy</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000182173/nico-adamczyk</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000525900/jan-stepniak</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Kacper Przybyłko</t>
+          <t>Krystian Kołodziejczak</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>952379</v>
+        <v>1516583</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>P. Niepolomice</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2005-02-05</t>
+          <t>2009-09-04</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1993-03-25</t>
+          <t>2009-01-01</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>91109529</v>
+        <v>2000525898</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>kacper-przybylko</t>
+          <t>krystian-kolodziejczak</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/91109529/kacper-przybylko</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000525898/krystian-kolodziejczak</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jan Stępniak</t>
+          <t>Sebastian Szczytniewski</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1516608</v>
+        <v>805499</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Internal transfer: Gornik Leczna II; date: 18/02/2026</t>
+          <t>Gornik Leczna</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2009-02-01</t>
+          <t>2003-03-19</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2009-01-01</t>
+          <t>2003-03-13</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2000525900</v>
+        <v>2000047883</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>jan-stepniak</t>
+          <t>sebastian-szczytniewski</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Gornik Leczna</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000525900/jan-stepniak</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000047883/sebastian-szczytniewski</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Krystian Kołodziejczak</t>
+          <t>Przemysław Misiak</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1516583</v>
+        <v>900848</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Gornik Leczna</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2009-09-04</t>
+          <t>2003-08-29</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2009-01-01</t>
+          <t>2003-08-23</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2000525898</v>
+        <v>96161668</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>krystian-kolodziejczak</t>
+          <t>przemyslaw-misiak</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Gornik Leczna</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000525898/krystian-kolodziejczak</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/96161668/przemyslaw-misiak</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sebastian Szczytniewski</t>
+          <t>Ederson</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>805499</v>
+        <v>238223</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Gornik Leczna</t>
+          <t>Fenerbahçe</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2003-03-19</t>
+          <t>1993-08-17</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2003-03-13</t>
+          <t>1999-07-07</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2000047883</v>
+        <v>19326796</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>sebastian-szczytniewski</t>
+          <t>ederson</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Atalanta BC</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000047883/sebastian-szczytniewski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/19326796/ederson</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Przemysław Misiak</t>
+          <t>Mohamed Touré</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>900848</v>
+        <v>742770</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Norwich</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2003-08-29</t>
+          <t>2004-03-26</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2003-08-23</t>
+          <t>2009-06-23</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>96161668</v>
+        <v>2000506639</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>przemyslaw-misiak</t>
+          <t>mohamed-force-toure</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Genoa CFC</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96161668/przemyslaw-misiak</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000506639/mohamed-force-toure</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mohamed Touré</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>742770</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2004-03-26</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2006-12-31</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>2000446784</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>mohamed-malang-toure</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Venezia FC</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000446784/mohamed-malang-toure</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Mohamed Touré</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>742770</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Norwich</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2004-03-26</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2006-01-22</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>2000241632</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>mohamed-toure</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>AC Carpi</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000241632/mohamed-toure</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Vitinha</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>487469</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PSG</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2000-02-13</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2000-03-15</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>83227945</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>vitinha</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Genoa CFC</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/83227945/vitinha</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Diego Gómez</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>996897</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Brighton</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2003-03-27</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1989-08-08</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>2000022020</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>diego-lopez-gomez</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Genoa CFC</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000022020/diego-lopez-gomez</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Idrissa Gueye</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>126665</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1989-09-26</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2006-09-16</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>12094946</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>idrissa-gueye</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Udinese Calcio</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/12094946/idrissa-gueye</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: add club paris-saint-germain from TM URL (2026-06-11)
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_dob_mismatch.xlsx
+++ b/data/sots_more_matches_dob_mismatch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1380,858 +1380,471 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Joan García</t>
+          <t>Kwasi Sibo</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>561613</v>
+        <v>538006</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2001-05-04</t>
+          <t>1998-06-24</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1991-03-29</t>
+          <t>1998-01-21</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2000065157</v>
+        <v>59130428</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>joan-garcia</t>
+          <t>kwasi-sibo</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>CA Osasuna</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000065157/joan-garcia</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/59130428/kwasi-sibo</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Kwasi Sibo</t>
+          <t>Liam Kelly</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>538006</v>
+        <v>208772</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Rangers</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1998-06-24</t>
+          <t>1996-01-23</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1998-01-21</t>
+          <t>1990-02-10</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>59130428</v>
+        <v>4001323</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>kwasi-sibo</t>
+          <t>liam-kelly</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Rotherham United</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/59130428/kwasi-sibo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/4001323/liam-kelly</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Liam Kelly</t>
+          <t>Mohamed Koné</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>208772</v>
+        <v>911985</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Rangers</t>
+          <t>R Charleroi SC</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1996-01-23</t>
+          <t>2002-03-07</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1990-02-10</t>
+          <t>2007-07-03</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4001323</v>
+        <v>12095721</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>liam-kelly</t>
+          <t>mohamed-kone</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Rotherham United</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/4001323/liam-kelly</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/12095721/mohamed-kone</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mohamed Koné</t>
+          <t>Rui Silva</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>911985</v>
+        <v>234811</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>R Charleroi SC</t>
+          <t>Sporting</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2002-03-07</t>
+          <t>1994-02-07</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2007-07-03</t>
+          <t>2007-02-28</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>12095721</v>
+        <v>2000526604</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>mohamed-kone</t>
+          <t>rui-silva</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Gil Vicente FC</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/12095721/mohamed-kone</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000526604/rui-silva</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mohamed Touré</t>
+          <t>Rui Silva</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>742770</v>
+        <v>234811</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Sporting</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2004-03-26</t>
+          <t>1994-02-07</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2009-06-23</t>
+          <t>1975-05-30</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2000506639</v>
+        <v>2000377975</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>mohamed-force-toure</t>
+          <t>rui-silva</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Genoa CFC</t>
+          <t>Gil Vicente FC</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000506639/mohamed-force-toure</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000377975/rui-silva</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mohamed Touré</t>
+          <t>Rui Silva</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>742770</v>
+        <v>234811</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Sporting</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2004-03-26</t>
+          <t>1994-02-07</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2006-12-31</t>
+          <t>1977-03-14</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2000446784</v>
+        <v>55003122</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>mohamed-malang-toure</t>
+          <t>rui-pedro-silva</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Venezia FC</t>
+          <t>Wolverhampton Wanderers</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000446784/mohamed-malang-toure</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/55003122/rui-pedro-silva</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mohamed Touré</t>
+          <t>Sander Berge</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>742770</v>
+        <v>333014</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Norwich</t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2004-03-26</t>
+          <t>1998-02-14</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2006-01-22</t>
+          <t>1998-02-18</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2000241632</v>
+        <v>53101282</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>mohamed-toure</t>
+          <t>sander-berge</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>AC Carpi</t>
+          <t>Fulham FC</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000241632/mohamed-toure</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/53101282/sander-berge</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pedro Neto</t>
+          <t>Roberto Fernández</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>487465</v>
+        <v>107318</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Cerro Porteño</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2000-03-09</t>
+          <t>1988-03-29</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1983-02-10</t>
+          <t>2002-07-03</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>736421</v>
+        <v>2000101543</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>pedro-neto</t>
+          <t>roberto-fernandez</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>SC Farense</t>
+          <t>RCD Espanyol Barcelona</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/736421/pedro-neto</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000101543/roberto-fernandez</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Rui Silva</t>
+          <t>Kealey Adamson</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>234811</v>
+        <v>1109828</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sporting</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1994-02-07</t>
+          <t>2003-02-17</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2007-02-28</t>
+          <t>2003-03-09</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>2000526604</v>
+        <v>2000090224</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>rui-silva</t>
+          <t>kealey-adamson</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Gil Vicente FC</t>
+          <t>Queens Park Rangers</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000526604/rui-silva</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000090224/kealey-adamson</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rui Silva</t>
+          <t>Justin Obikwu</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>234811</v>
+        <v>873270</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Sporting</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1994-02-07</t>
+          <t>2004-05-06</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1975-05-30</t>
+          <t>2004-02-18</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2000377975</v>
+        <v>2000131091</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>rui-silva</t>
+          <t>justin-obikwu</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Gil Vicente FC</t>
+          <t>Queens Park Rangers</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000377975/rui-silva</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000131091/justin-obikwu</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Rui Silva</t>
+          <t>Mika Mármol</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>234811</v>
+        <v>617060</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Sporting</t>
+          <t>UD Las Palmas</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1994-02-07</t>
+          <t>2001-07-02</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1977-03-14</t>
+          <t>2001-07-01</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>55003122</v>
+        <v>67295761</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>rui-pedro-silva</t>
+          <t>mika-marmol</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Wolverhampton Wanderers</t>
+          <t>UD Las Palmas</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/55003122/rui-pedro-silva</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Sander Berge</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>333014</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Fulham</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>1998-02-14</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>1998-02-18</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>53101282</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>sander-berge</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Fulham FC</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/53101282/sander-berge</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Vitinha</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>487469</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>PSG</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>2000-02-13</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2000-03-15</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>83227945</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>vitinha</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Genoa CFC</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/83227945/vitinha</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Alfie Jones</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>340990</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Middlesbrough</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>1997-10-07</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2008-12-06</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>2000506253</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>alfie-jones</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Swansea City</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000506253/alfie-jones</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Diego Gómez</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>996897</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Brighton</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2003-03-27</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>1989-08-08</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>2000022020</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>diego-lopez-gomez</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Genoa CFC</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000022020/diego-lopez-gomez</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Idrissa Gueye</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>126665</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Everton</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>1989-09-26</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>2006-09-16</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>12094946</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>idrissa-gueye</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Udinese Calcio</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/12094946/idrissa-gueye</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Roberto Fernández</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>107318</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Cerro Porteño</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>1988-03-29</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2002-07-03</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>2000101543</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>roberto-fernandez</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>RCD Espanyol Barcelona</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000101543/roberto-fernandez</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Kealey Adamson</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1109828</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>QPR</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>2003-02-17</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2003-03-09</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>2000090224</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>kealey-adamson</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Queens Park Rangers</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000090224/kealey-adamson</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Justin Obikwu</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>873270</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>QPR</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2004-05-06</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2004-02-18</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>2000131091</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>justin-obikwu</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Queens Park Rangers</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000131091/justin-obikwu</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Mika Mármol</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>617060</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>UD Las Palmas</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2001-07-02</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2001-07-01</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>67295761</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>mika-marmol</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>UD Las Palmas</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
         <is>
           <t>https://sortitoutsi.net/football-manager-2026/person/67295761/mika-marmol</t>
         </is>

</xml_diff>

<commit_message>
auto: add club real-madrid from TM URL (2026-07-14)
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_dob_mismatch.xlsx
+++ b/data/sots_more_matches_dob_mismatch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1420,6 +1420,49 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Javi Navarro</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1328089</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>RM Castilla</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2007-01-25</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1982-11-18</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>67182931</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>javi-navarro</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Levante UD</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://sortitoutsi.net/football-manager-2026/person/67182931/javi-navarro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>